<commit_message>
feat: queda de receita (Fase 5): REVENUE_DROP mensal via taxa-map, regra P1 e aba na tela de receitas
Motor: receita da casa por carteira = PL x taxa anual / 12, calculada no
normalize so no periodo mensal a partir do taxa-map da instancia
(taxa-map.local.json sobre taxa-map.json, padrao do class-map). Diff emite
REVENUE_DROP quando a queda passa de 5% (percentual puro, sem piso), com
evidencias e materialidade. Regra de oportunidade queda-receita P1 com
prazo de 15 dias. Fixtures desenham a queda em GAMA (-6,25% exato, sem
disparar outros eventos); round-trip e CLI real confirmam 4 eventos no
mensal. Tela: aba Queda de receita dentro de Receitas & ROA, com cortes de
casa/gerente/carteira, filtro de assessor, CSV e deep link. Rentabilidade
do cliente fica fora do evento (metrica propria do fluxo mensal).
Revisor: 1 P1 corrigido (downloadCSV), 2 P2 aplicados.

Co-Authored-By: Claude <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/audit-engine/tests/fixtures-sinteticos/mensais/posicao-2026-06.xlsx
+++ b/audit-engine/tests/fixtures-sinteticos/mensais/posicao-2026-06.xlsx
@@ -868,10 +868,10 @@
         <v>8</v>
       </c>
       <c r="C8">
-        <v>256000</v>
+        <v>216000</v>
       </c>
       <c r="D8">
-        <v>256000</v>
+        <v>216000</v>
       </c>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.25">
@@ -882,10 +882,10 @@
         <v>4</v>
       </c>
       <c r="C9">
-        <v>256000</v>
+        <v>216000</v>
       </c>
       <c r="D9">
-        <v>256000</v>
+        <v>216000</v>
       </c>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.25">
@@ -893,10 +893,10 @@
         <v>15</v>
       </c>
       <c r="C10">
-        <v>640000</v>
+        <v>600000</v>
       </c>
       <c r="D10">
-        <v>640000</v>
+        <v>600000</v>
       </c>
     </row>
   </sheetData>

</xml_diff>